<commit_message>
Concilia backlogs tras el PR #21 y sube el cierre del Sprint 2
Sprint 2: restaura la versión oficial de cierre del 06-10-2026 (30 tareas, 92 h reales), la misma del Drive. Sprint 3: agrega las tareas arrastradas de FS-HU-04 y FS-HU-15 (SMTP). Product Backlog: FS-HU-04 en el Sprint 3. Agrega el Documento del Sprint Backlog 2, el Documento validando, los burndown y su plantilla; Guía 2.4 y control con el cierre del Sprint 2.
</commit_message>
<xml_diff>
--- a/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/control-capstone-2026-FitSearch.xlsx
+++ b/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/control-capstone-2026-FitSearch.xlsx
@@ -928,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A4:J19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.1484375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="22" min="1" max="2"/>
@@ -942,6 +942,9 @@
     <col width="35" customWidth="1" style="22" min="10" max="10"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="23">
       <c r="A4" s="39" t="inlineStr">
         <is>
@@ -1358,7 +1361,7 @@
       <c r="I12" s="43" t="n"/>
       <c r="J12" s="43" t="inlineStr">
         <is>
-          <t>Sprint 1: 11 tareas, 43 h estimadas y 43 h reales (Luis 15, Rodrigo 14, Nicolás 14). Documento Validando Sprint 1 completo con avances día a día, gráfico de avance y pila del producto actualizada; el Product Owner aceptó FS-HU-01 y FS-HU-02 el 24-09-2026 (columna A/R, con observaciones) y la retrospectiva quedó registrada el 24-09-2026; Luis Méndez aprobó la revisión posterior del código (PR #6) el 24-09-2026; Sprint 1 cerrado. Sprint 2: borrador con 23 tareas en 'Sprint 2/PMOInformatica_Plantilla_de_Sprint_Backlog.xlsx'; horas estimadas y responsables pendientes de la planificación del equipo. Sprint 2: el 03-10-2026 Luis Méndez aprobó la revisión de código de FS-HU-02 y FS-HU-15 a FS-HU-20 (PR #9; 2 h junto con el PR #10) y el Product Owner aceptó esas historias y FS-HU-03 (revisada en el PR #8); falta que el equipo registre sus horas reales del sprint y el Documento Validando Sprint 2.</t>
+          <t>Sprint 1: 11 tareas, 43 h estimadas y 43 h reales (Luis 15, Rodrigo 14, Nicolás 14). Documento Validando Sprint 1 completo con avances día a día, gráfico de avance y pila del producto actualizada; el Product Owner aceptó FS-HU-01 y FS-HU-02 el 24-09-2026 (columna A/R, con observaciones) y la retrospectiva quedó registrada el 24-09-2026; Luis Méndez aprobó la revisión posterior del código (PR #6) el 24-09-2026; Sprint 1 cerrado. Sprint 2: cerrado el 04-10-2026 con 30 tareas, 110 h estimadas y 92 h reales (Rodrigo Cárcamo Rojas 51, Nicolás Silva 23 y Luis Méndez 18), registradas al cierre según el trabajo entregado en GitHub; Documento Sprint Backlog 2, Documento Validando Sprint 2 y burndown del Sprint 2 en 'Sprint 2/'. El Product Owner aceptó FS-HU-02 (tipo de cuenta), FS-HU-03 y FS-HU-15 a FS-HU-20 el 03-10-2026; FS-HU-04 (PR #11 en corrección) y FS-HU-13 pasan al Sprint 3. Sprint 3: borrador en 'Sprint 3/', planificación pendiente.</t>
         </is>
       </c>
     </row>
@@ -1496,13 +1499,13 @@
       </c>
       <c r="H15" s="44" t="inlineStr">
         <is>
-          <t>No Iniciado</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="I15" s="43" t="n"/>
       <c r="J15" s="43" t="inlineStr">
         <is>
-          <t>Plantilla lista con la identificación del Sprint 1; la completan Luis Méndez y Nicolás Silva en la reunión retrospectiva (el Product Owner no asiste).</t>
+          <t>Sprint 1: retrospectiva escrita (asíncrona) registrada el 24-09-2026 en 'Sprint 1/Plantilla_Resumen_Reunion_Retrospectiva.docx', con las respuestas de los tres integrantes. Sprint 2: pendiente de las respuestas del equipo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Retrospectiva del Sprint 2, horas y documento del Sprint Backlog 3 con burndown, diario de Nicolas renombrado y planilla duplicada eliminada
</commit_message>
<xml_diff>
--- a/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/control-capstone-2026-FitSearch.xlsx
+++ b/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/control-capstone-2026-FitSearch.xlsx
@@ -1358,7 +1358,7 @@
       <c r="I12" s="43" t="n"/>
       <c r="J12" s="43" t="inlineStr">
         <is>
-          <t>Sprint 1: 11 tareas, 43 h estimadas y 43 h reales (Luis 15, Rodrigo 14, Nicolás 14). Documento Validando Sprint 1 completo con avances día a día, gráfico de avance y pila del producto actualizada; el Product Owner aceptó FS-HU-01 y FS-HU-02 el 24-09-2026 (columna A/R, con observaciones) y la retrospectiva quedó registrada el 24-09-2026; Luis Méndez aprobó la revisión posterior del código (PR #6) el 24-09-2026; Sprint 1 cerrado. Sprint 2: cerrado el 04-10-2026 con 30 tareas, 110 h estimadas y 92 h reales (Rodrigo Cárcamo Rojas 51, Nicolás Silva 23 y Luis Méndez 18), registradas al cierre según el trabajo entregado en GitHub; Documento Sprint Backlog 2, Documento Validando Sprint 2 y burndown del Sprint 2 en 'Sprint 2/'. El Product Owner aceptó FS-HU-02 (tipo de cuenta), FS-HU-03 y FS-HU-15 a FS-HU-20 el 03-10-2026; FS-HU-04 (PR #11 en corrección) y FS-HU-13 pasan al Sprint 3. Sprint 3 (desde el 05-10-2026): el Sprint Backlog 3 registra las tareas implementadas de FS-HU-04, FS-HU-05, FS-HU-06, FS-HU-12, FS-HU-13, FS-HU-14 y FS-HU-21 a FS-HU-24, y la configuración del SMTP de FS-HU-15. El Product Owner aceptó FS-HU-04 el 12-10-2026; las demás siguen pendientes de aceptación. Las horas reales del Sprint 3 aún no se registran.</t>
+          <t>Sprint 1: 11 tareas, 43 h estimadas y 43 h reales (Luis 15, Rodrigo 14, Nicolás 14). Documento Validando Sprint 1 completo con avances día a día, gráfico de avance y pila del producto actualizada; el Product Owner aceptó FS-HU-01 y FS-HU-02 el 24-09-2026 (columna A/R, con observaciones) y la retrospectiva quedó registrada el 24-09-2026; Luis Méndez aprobó la revisión posterior del código (PR #6) el 24-09-2026; Sprint 1 cerrado. Sprint 2: cerrado el 04-10-2026 con 30 tareas, 110 h estimadas y 92 h reales (Rodrigo Cárcamo Rojas 51, Nicolás Silva 23 y Luis Méndez 18), registradas al cierre según el trabajo entregado en GitHub; Documento Sprint Backlog 2, Documento Validando Sprint 2 y burndown del Sprint 2 en 'Sprint 2/'. El Product Owner aceptó FS-HU-02 (tipo de cuenta), FS-HU-03 y FS-HU-15 a FS-HU-20 el 03-10-2026; FS-HU-04 (PR #11 en corrección) y FS-HU-13 pasan al Sprint 3. Sprint 3 (desde el 05-10-2026): el Sprint Backlog 3 registra las tareas implementadas de FS-HU-04, FS-HU-05, FS-HU-06, FS-HU-12, FS-HU-13, FS-HU-14 y FS-HU-21 a FS-HU-24, y la configuración del SMTP de FS-HU-15. El Product Owner aceptó FS-HU-04 el 12-10-2026; las demás siguen pendientes de aceptación. Horas del Sprint 3 registradas el 12-10-2026 según el trabajo entregado en GitHub: 32 tareas, 97 h estimadas y 95 h registradas al día 8 (Rodrigo Cárcamo Rojas 52, Luis Méndez 40 y Nicolás Silva 3); Documento Sprint Backlog 3 y burndown del Sprint 3 en 'Sprint 3/'.</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       <c r="I15" s="43" t="n"/>
       <c r="J15" s="43" t="inlineStr">
         <is>
-          <t>Sprint 1: retrospectiva escrita (asíncrona) registrada el 24-09-2026 en 'Sprint 1/Plantilla_Resumen_Reunion_Retrospectiva.docx', con las respuestas de los tres integrantes. Sprint 2: pendiente de las respuestas del equipo.</t>
+          <t>Sprint 1: retrospectiva escrita (asíncrona) registrada el 24-09-2026 en 'Sprint 1/Plantilla_Resumen_Reunion_Retrospectiva.docx', con las respuestas de los tres integrantes. Sprint 2: retrospectiva escrita (asíncrona) registrada el 12-10-2026 en 'Sprint 2/Plantilla_Resumen_Reunion_Retrospectiva.docx', con las respuestas de los tres integrantes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Defectos 27 y 29: el mapa se recupera si falla el estilo y sus controles estan en espanol
</commit_message>
<xml_diff>
--- a/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/control-capstone-2026-FitSearch.xlsx
+++ b/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/control-capstone-2026-FitSearch.xlsx
@@ -1549,7 +1549,7 @@
       <c r="I16" s="43" t="n"/>
       <c r="J16" s="43" t="inlineStr">
         <is>
-          <t>Planilla de Casos de Prueba: 80 casos (CP-001 a CP-080), 77 aprobados y 3 sin ejecutar (CP-024 y CP-025, acceso con Google; CP-078, mapa real en main). Registro de Defectos con 29 defectos: 26 corregidos y 3 abiertos (27 a 29, del mapa nuevo del PR #27). El 15-10-2026 se repitieron CP-076 y CP-077 con MapLibre (189/189 en el frontend); CP-078 sigue pendiente con el mapa nuevo. Comprobaciones con MySQL real: npm run test:mysql:agenda, 55/55 sobre main 662e79c el 12-10-2026. Evidencias en FASE 2/Evidencias Proyecto/Evidencias de documentación/Sprint N/Capturas del sistema. 19-10-2026: CP-081 a CP-087 (mejoras de interfaz, SC-19), todos aprobados → 87 casos, 84 aprobados y 3 sin ejecutar (CP-024, CP-025 y CP-078); defectos 30 a 34 corregidos → 34 defectos: 31 corregidos y 3 abiertos (27 a 29). Evidencias en Plan de Pruebas/Mejoras_Interfaz_2026-10-19*. 19-10-2026 (SC-20, reserva con calendario): CP-088 a CP-091 aprobados → 91 casos, 88 aprobados y 3 sin ejecutar. Evidencias en Plan de Pruebas/Flujo_Reservas_2026-10-19*. SC-21 (calendario al publicar horarios): CP-092 y CP-093 aprobados → 93 casos, 90 aprobados y 3 sin ejecutar. Evidencias en Plan de Pruebas/Publicar_Horario_2026-10-19*. Defecto 35 (mapa que se veía de lejos por una ubicación fuera de Chile) corregido con CP-094 → 94 casos, 91 aprobados y 3 sin ejecutar; 35 defectos: 32 corregidos y 3 abiertos. Evidencias en Plan de Pruebas/Mapa_Chile_2026-10-19*. SC-22 (detalle del profesional en el mapa): CP-095 y CP-096 aprobados y defecto 28 corregido → 96 casos, 93 aprobados y 3 sin ejecutar; 35 defectos: 33 corregidos y 2 abiertos (27 y 29). Evidencias en Plan de Pruebas/Detalle_Mapa_2026-10-19*. SC-23 (buscador general del Inicio): CP-097 y CP-098 aprobados → 98 casos, 95 aprobados y 3 sin ejecutar. Evidencias en Plan de Pruebas/Buscador_Inicio_2026-10-19*. SC-24 (dirección de atención y coordenadas en Chile en la ficha profesional): CP-099 y CP-100 aprobados → 100 casos, 97 aprobados y 3 sin ejecutar. Evidencias en Plan de Pruebas/Direccion_Ficha_2026-10-19*.</t>
+          <t>Planilla de Casos de Prueba: 80 casos (CP-001 a CP-080), 77 aprobados y 3 sin ejecutar (CP-024 y CP-025, acceso con Google; CP-078, mapa real en main). Registro de Defectos con 29 defectos: 26 corregidos y 3 abiertos (27 a 29, del mapa nuevo del PR #27). El 15-10-2026 se repitieron CP-076 y CP-077 con MapLibre (189/189 en el frontend); CP-078 sigue pendiente con el mapa nuevo. Comprobaciones con MySQL real: npm run test:mysql:agenda, 55/55 sobre main 662e79c el 12-10-2026. Evidencias en FASE 2/Evidencias Proyecto/Evidencias de documentación/Sprint N/Capturas del sistema. 19-10-2026: CP-081 a CP-087 (mejoras de interfaz, SC-19), todos aprobados → 87 casos, 84 aprobados y 3 sin ejecutar (CP-024, CP-025 y CP-078); defectos 30 a 34 corregidos → 34 defectos: 31 corregidos y 3 abiertos (27 a 29). Evidencias en Plan de Pruebas/Mejoras_Interfaz_2026-10-19*. 19-10-2026 (SC-20, reserva con calendario): CP-088 a CP-091 aprobados → 91 casos, 88 aprobados y 3 sin ejecutar. Evidencias en Plan de Pruebas/Flujo_Reservas_2026-10-19*. SC-21 (calendario al publicar horarios): CP-092 y CP-093 aprobados → 93 casos, 90 aprobados y 3 sin ejecutar. Evidencias en Plan de Pruebas/Publicar_Horario_2026-10-19*. Defecto 35 (mapa que se veía de lejos por una ubicación fuera de Chile) corregido con CP-094 → 94 casos, 91 aprobados y 3 sin ejecutar; 35 defectos: 32 corregidos y 3 abiertos. Evidencias en Plan de Pruebas/Mapa_Chile_2026-10-19*. SC-22 (detalle del profesional en el mapa): CP-095 y CP-096 aprobados y defecto 28 corregido → 96 casos, 93 aprobados y 3 sin ejecutar; 35 defectos: 33 corregidos y 2 abiertos (27 y 29). Evidencias en Plan de Pruebas/Detalle_Mapa_2026-10-19*. SC-23 (buscador general del Inicio): CP-097 y CP-098 aprobados → 98 casos, 95 aprobados y 3 sin ejecutar. Evidencias en Plan de Pruebas/Buscador_Inicio_2026-10-19*. SC-24 (dirección de atención y coordenadas en Chile en la ficha profesional): CP-099 y CP-100 aprobados → 100 casos, 97 aprobados y 3 sin ejecutar. Evidencias en Plan de Pruebas/Direccion_Ficha_2026-10-19*. 21-10-2026: corregidos los defectos 27 y 29 del mapa (CP-101 y CP-102 aprobados) → 102 casos, 99 aprobados y 3 sin ejecutar; 35 defectos, todos corregidos. Evidencias en Plan de Pruebas/Defectos_Mapa_2026-10-21*.</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2259,7 @@
       <c r="F22" s="43" t="n"/>
       <c r="G22" s="43" t="inlineStr">
         <is>
-          <t>Sprint 1: pruebas unitarias y de componentes con Jest (backend) y Vitest (frontend), todas aprobadas. Al 15-10-2026: 233 pruebas en el backend y 189 en el frontend, todas aprobadas. Al 19-10-2026: 241 en el backend y 231 en el frontend (mejoras de interfaz, SC-19; reserva con calendario, SC-20, y calendario al publicar horarios, SC-21; mapa limitado a Chile, defecto 35; detalle en el mapa, SC-22; buscador general, SC-23; dirección del profesional, SC-24), todas aprobadas.</t>
+          <t>Sprint 1: pruebas unitarias y de componentes con Jest (backend) y Vitest (frontend), todas aprobadas. Al 15-10-2026: 233 pruebas en el backend y 189 en el frontend, todas aprobadas. Al 19-10-2026: 241 en el backend y 231 en el frontend (mejoras de interfaz, SC-19; reserva con calendario, SC-20, y calendario al publicar horarios, SC-21; mapa limitado a Chile, defecto 35; detalle en el mapa, SC-22; buscador general, SC-23; dirección del profesional, SC-24), todas aprobadas. Al 21-10-2026: 241 en el backend y 233 en el frontend (defectos 27 y 29 del mapa), todas aprobadas.</t>
         </is>
       </c>
     </row>

</xml_diff>